<commit_message>
Curva S actualizada 2026-07-09 17:36 Chile
</commit_message>
<xml_diff>
--- a/data/50001546 - XEMORTIZ.xlsx
+++ b/data/50001546 - XEMORTIZ.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1762" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1763" uniqueCount="388">
   <si>
     <t>50001546 - XEMORTIZ</t>
   </si>
@@ -630,6 +630,9 @@
     <t>Control de calidad corte laser ,Recepcion materiales corte laser</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1214777626758318</t>
   </si>
   <si>
@@ -643,9 +646,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bodega:,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214777626772872</t>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46209.63604493055</v>
+        <v>46212.88596806713</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>197</v>
@@ -4967,30 +4967,34 @@
       <c r="R56" s="6"/>
       <c r="S56" s="6"/>
       <c r="T56" s="6"/>
-      <c r="U56" s="6"/>
+      <c r="U56" s="12" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B57" s="8">
         <v>46155.60612483796</v>
       </c>
-      <c r="C57" s="9"/>
+      <c r="C57" s="8">
+        <v>46212.8859408912</v>
+      </c>
       <c r="D57" s="8">
-        <v>46205.60920457176</v>
+        <v>46212.88596140046</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I57" s="8">
         <v>46202</v>
@@ -5014,7 +5018,7 @@
         <v>134</v>
       </c>
       <c r="P57" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q57" s="8">
         <v>46202</v>
@@ -5026,10 +5030,10 @@
         <v>32</v>
       </c>
       <c r="T57" s="9">
-        <v>0</v>
-      </c>
-      <c r="U57" s="12" t="s">
-        <v>204</v>
+        <v>1</v>
+      </c>
+      <c r="U57" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -5043,7 +5047,7 @@
         <v>46209.63603707176</v>
       </c>
       <c r="D58" s="5">
-        <v>46209.63605303241</v>
+        <v>46212.88595888889</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>206</v>
@@ -5115,10 +5119,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I59" s="8">
         <v>46202</v>
@@ -5157,7 +5161,7 @@
         <v>0</v>
       </c>
       <c r="U59" s="12" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5230,9 +5234,11 @@
       <c r="B61" s="8">
         <v>46155.606156319445</v>
       </c>
-      <c r="C61" s="9"/>
+      <c r="C61" s="8">
+        <v>46212.886193530096</v>
+      </c>
       <c r="D61" s="8">
-        <v>46212.16840913195</v>
+        <v>46212.88631315972</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>216</v>
@@ -5241,10 +5247,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I61" s="8">
         <v>46211</v>
@@ -5280,10 +5286,10 @@
         <v>218</v>
       </c>
       <c r="T61" s="9">
-        <v>0</v>
-      </c>
-      <c r="U61" s="12" t="s">
-        <v>204</v>
+        <v>1</v>
+      </c>
+      <c r="U61" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5293,9 +5299,11 @@
       <c r="B62" s="5">
         <v>46155.60616390046</v>
       </c>
-      <c r="C62" s="6"/>
+      <c r="C62" s="5">
+        <v>46212.886227650466</v>
+      </c>
       <c r="D62" s="5">
-        <v>46209.1697228125</v>
+        <v>46212.8864002662</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>217</v>
@@ -5343,10 +5351,10 @@
         <v>218</v>
       </c>
       <c r="T62" s="6">
-        <v>0</v>
-      </c>
-      <c r="U62" s="10" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="U62" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5468,7 +5476,7 @@
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46209.636044467596</v>
+        <v>46212.88623596064</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>228</v>
@@ -5521,7 +5529,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46209.63604388889</v>
+        <v>46212.88623552083</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>228</v>
@@ -5574,7 +5582,7 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46209.63604545139</v>
+        <v>46212.88623635417</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>228</v>
@@ -5627,7 +5635,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46209.63604590278</v>
+        <v>46212.88623675926</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>228</v>
@@ -5680,7 +5688,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46209.636043402774</v>
+        <v>46212.886234907404</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>228</v>
@@ -6447,10 +6455,10 @@
         <v>26</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I83" s="9"/>
       <c r="J83" s="8">
@@ -6508,10 +6516,10 @@
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I84" s="5">
         <v>46164</v>
@@ -6550,7 +6558,7 @@
         <v>0</v>
       </c>
       <c r="U84" s="12" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -6571,10 +6579,10 @@
         <v>26</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H85" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I85" s="8">
         <v>46197</v>
@@ -6613,7 +6621,7 @@
         <v>0</v>
       </c>
       <c r="U85" s="12" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -6634,10 +6642,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I86" s="5">
         <v>46231</v>
@@ -6676,7 +6684,7 @@
         <v>0</v>
       </c>
       <c r="U86" s="12" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-26 15:38 UTC
</commit_message>
<xml_diff>
--- a/data/50001546 - XEMORTIZ.xlsx
+++ b/data/50001546 - XEMORTIZ.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1767" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1768" uniqueCount="387">
   <si>
     <t>50001546 - XEMORTIZ</t>
   </si>
@@ -5415,9 +5415,11 @@
       <c r="B63" s="8">
         <v>46155.60617082176</v>
       </c>
-      <c r="C63" s="9"/>
+      <c r="C63" s="8">
+        <v>46260.64293943287</v>
+      </c>
       <c r="D63" s="8">
-        <v>46260.579079814815</v>
+        <v>46260.64295446759</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>220</v>
@@ -5452,7 +5454,9 @@
       <c r="Q63" s="9"/>
       <c r="R63" s="9"/>
       <c r="S63" s="9"/>
-      <c r="T63" s="9"/>
+      <c r="T63" s="9">
+        <v>1</v>
+      </c>
       <c r="U63" s="11" t="s">
         <v>33</v>
       </c>
@@ -6795,7 +6799,7 @@
       </c>
       <c r="C87" s="9"/>
       <c r="D87" s="8">
-        <v>46258.57700428241</v>
+        <v>46260.64235780093</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>270</v>
@@ -6831,7 +6835,9 @@
       <c r="R87" s="9"/>
       <c r="S87" s="9"/>
       <c r="T87" s="9"/>
-      <c r="U87" s="9"/>
+      <c r="U87" s="12" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
@@ -8508,9 +8514,11 @@
       <c r="B118" s="5">
         <v>46155.60664190972</v>
       </c>
-      <c r="C118" s="6"/>
+      <c r="C118" s="5">
+        <v>46260.6423377662</v>
+      </c>
       <c r="D118" s="5">
-        <v>46260.579217418985</v>
+        <v>46260.642349120375</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>328</v>
@@ -8558,10 +8566,10 @@
         <v>32</v>
       </c>
       <c r="T118" s="6">
-        <v>0</v>
-      </c>
-      <c r="U118" s="11" t="s">
-        <v>33</v>
+        <v>1</v>
+      </c>
+      <c r="U118" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
@@ -8571,9 +8579,11 @@
       <c r="B119" s="8">
         <v>46155.60665081019</v>
       </c>
-      <c r="C119" s="9"/>
+      <c r="C119" s="8">
+        <v>46260.64231520833</v>
+      </c>
       <c r="D119" s="8">
-        <v>46258.57706458333</v>
+        <v>46260.64231946759</v>
       </c>
       <c r="E119" s="9" t="s">
         <v>190</v>
@@ -8622,9 +8632,11 @@
       <c r="B120" s="5">
         <v>46155.60665825232</v>
       </c>
-      <c r="C120" s="6"/>
+      <c r="C120" s="5">
+        <v>46260.642316087964</v>
+      </c>
       <c r="D120" s="5">
-        <v>46258.57706256944</v>
+        <v>46260.64231998843</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>190</v>
@@ -8673,9 +8685,11 @@
       <c r="B121" s="8">
         <v>46155.60666534722</v>
       </c>
-      <c r="C121" s="9"/>
+      <c r="C121" s="8">
+        <v>46260.64231671296</v>
+      </c>
       <c r="D121" s="8">
-        <v>46258.57706253472</v>
+        <v>46260.64232047454</v>
       </c>
       <c r="E121" s="9" t="s">
         <v>190</v>
@@ -8724,9 +8738,11 @@
       <c r="B122" s="5">
         <v>46155.60667253472</v>
       </c>
-      <c r="C122" s="6"/>
+      <c r="C122" s="5">
+        <v>46260.642317199075</v>
+      </c>
       <c r="D122" s="5">
-        <v>46258.577062592594</v>
+        <v>46260.64232087963</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>190</v>
@@ -8775,9 +8791,11 @@
       <c r="B123" s="8">
         <v>46155.63591585648</v>
       </c>
-      <c r="C123" s="9"/>
+      <c r="C123" s="8">
+        <v>46260.64231782407</v>
+      </c>
       <c r="D123" s="8">
-        <v>46258.57706246528</v>
+        <v>46260.6423212963</v>
       </c>
       <c r="E123" s="9" t="s">
         <v>190</v>
@@ -8828,7 +8846,7 @@
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="5">
-        <v>46155.60689462963</v>
+        <v>46260.642775</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>338</v>
@@ -8875,7 +8893,7 @@
       </c>
       <c r="C125" s="9"/>
       <c r="D125" s="8">
-        <v>46246.192134826386</v>
+        <v>46260.64234953704</v>
       </c>
       <c r="E125" s="9" t="s">
         <v>341</v>
@@ -8936,7 +8954,7 @@
       </c>
       <c r="C126" s="6"/>
       <c r="D126" s="5">
-        <v>46245.16770908565</v>
+        <v>46260.642328622685</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>190</v>
@@ -8987,7 +9005,7 @@
       </c>
       <c r="C127" s="9"/>
       <c r="D127" s="8">
-        <v>46245.16771032407</v>
+        <v>46260.642331759256</v>
       </c>
       <c r="E127" s="9" t="s">
         <v>190</v>
@@ -9038,7 +9056,7 @@
       </c>
       <c r="C128" s="6"/>
       <c r="D128" s="5">
-        <v>46245.16773751157</v>
+        <v>46260.642328773145</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>190</v>
@@ -9089,7 +9107,7 @@
       </c>
       <c r="C129" s="9"/>
       <c r="D129" s="8">
-        <v>46245.16774123843</v>
+        <v>46260.64233192129</v>
       </c>
       <c r="E129" s="9" t="s">
         <v>190</v>
@@ -9140,7 +9158,7 @@
       </c>
       <c r="C130" s="6"/>
       <c r="D130" s="5">
-        <v>46245.16769219907</v>
+        <v>46260.642331875</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>190</v>
@@ -9189,9 +9207,11 @@
       <c r="B131" s="8">
         <v>46155.60671987268</v>
       </c>
-      <c r="C131" s="9"/>
+      <c r="C131" s="8">
+        <v>46260.64265844907</v>
+      </c>
       <c r="D131" s="8">
-        <v>46260.57928197917</v>
+        <v>46260.64267006944</v>
       </c>
       <c r="E131" s="9" t="s">
         <v>353</v>
@@ -9239,10 +9259,10 @@
         <v>32</v>
       </c>
       <c r="T131" s="9">
-        <v>0</v>
-      </c>
-      <c r="U131" s="11" t="s">
-        <v>33</v>
+        <v>1</v>
+      </c>
+      <c r="U131" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
@@ -9252,9 +9272,11 @@
       <c r="B132" s="5">
         <v>46155.60672658565</v>
       </c>
-      <c r="C132" s="6"/>
+      <c r="C132" s="5">
+        <v>46260.64242549769</v>
+      </c>
       <c r="D132" s="5">
-        <v>46246.1681611574</v>
+        <v>46260.64242690972</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>190</v>
@@ -9305,9 +9327,11 @@
       <c r="B133" s="8">
         <v>46155.60673355324</v>
       </c>
-      <c r="C133" s="9"/>
+      <c r="C133" s="8">
+        <v>46260.6424750463</v>
+      </c>
       <c r="D133" s="8">
-        <v>46246.16816508102</v>
+        <v>46260.64247767361</v>
       </c>
       <c r="E133" s="9" t="s">
         <v>190</v>
@@ -9358,9 +9382,11 @@
       <c r="B134" s="5">
         <v>46155.60674053241</v>
       </c>
-      <c r="C134" s="6"/>
+      <c r="C134" s="5">
+        <v>46260.64252721065</v>
+      </c>
       <c r="D134" s="5">
-        <v>46246.16816266204</v>
+        <v>46260.642528993056</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>190</v>
@@ -9411,9 +9437,11 @@
       <c r="B135" s="8">
         <v>46155.60674741898</v>
       </c>
-      <c r="C135" s="9"/>
+      <c r="C135" s="8">
+        <v>46260.64259072917</v>
+      </c>
       <c r="D135" s="8">
-        <v>46246.16816386574</v>
+        <v>46260.642592013886</v>
       </c>
       <c r="E135" s="9" t="s">
         <v>190</v>
@@ -9464,9 +9492,11 @@
       <c r="B136" s="5">
         <v>46155.63830266204</v>
       </c>
-      <c r="C136" s="6"/>
+      <c r="C136" s="5">
+        <v>46260.64264464121</v>
+      </c>
       <c r="D136" s="5">
-        <v>46246.16811372685</v>
+        <v>46260.64264611111</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>190</v>
@@ -9515,9 +9545,11 @@
       <c r="B137" s="8">
         <v>46155.60675400463</v>
       </c>
-      <c r="C137" s="9"/>
+      <c r="C137" s="8">
+        <v>46260.64276806713</v>
+      </c>
       <c r="D137" s="8">
-        <v>46260.57930319445</v>
+        <v>46260.64277840278</v>
       </c>
       <c r="E137" s="9" t="s">
         <v>362</v>
@@ -9565,10 +9597,10 @@
         <v>32</v>
       </c>
       <c r="T137" s="9">
-        <v>0</v>
-      </c>
-      <c r="U137" s="11" t="s">
-        <v>33</v>
+        <v>1</v>
+      </c>
+      <c r="U137" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="138" spans="1:21" x14ac:dyDescent="0.25">
@@ -9578,9 +9610,11 @@
       <c r="B138" s="5">
         <v>46155.60676105324</v>
       </c>
-      <c r="C138" s="6"/>
+      <c r="C138" s="5">
+        <v>46260.642747453705</v>
+      </c>
       <c r="D138" s="5">
-        <v>46247.167744872684</v>
+        <v>46260.64275222222</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>190</v>
@@ -9629,9 +9663,11 @@
       <c r="B139" s="8">
         <v>46155.60677012731</v>
       </c>
-      <c r="C139" s="9"/>
+      <c r="C139" s="8">
+        <v>46260.642748495375</v>
+      </c>
       <c r="D139" s="8">
-        <v>46247.16774606481</v>
+        <v>46260.642752685184</v>
       </c>
       <c r="E139" s="9" t="s">
         <v>190</v>
@@ -9680,9 +9716,11 @@
       <c r="B140" s="5">
         <v>46155.60681737268</v>
       </c>
-      <c r="C140" s="6"/>
+      <c r="C140" s="5">
+        <v>46260.642749328705</v>
+      </c>
       <c r="D140" s="5">
-        <v>46247.16774079861</v>
+        <v>46260.642753148146</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>190</v>
@@ -9731,9 +9769,11 @@
       <c r="B141" s="8">
         <v>46155.60682548611</v>
       </c>
-      <c r="C141" s="9"/>
+      <c r="C141" s="8">
+        <v>46260.64275002315</v>
+      </c>
       <c r="D141" s="8">
-        <v>46247.16774200232</v>
+        <v>46260.642753576394</v>
       </c>
       <c r="E141" s="9" t="s">
         <v>190</v>
@@ -9782,9 +9822,11 @@
       <c r="B142" s="5">
         <v>46155.63928425926</v>
       </c>
-      <c r="C142" s="6"/>
+      <c r="C142" s="5">
+        <v>46260.64275072917</v>
+      </c>
       <c r="D142" s="5">
-        <v>46247.16771978009</v>
+        <v>46260.64275396991</v>
       </c>
       <c r="E142" s="6" t="s">
         <v>190</v>
@@ -9898,7 +9940,7 @@
       </c>
       <c r="C144" s="6"/>
       <c r="D144" s="5">
-        <v>46248.168570243055</v>
+        <v>46260.64276216435</v>
       </c>
       <c r="E144" s="6" t="s">
         <v>190</v>
@@ -9949,7 +9991,7 @@
       </c>
       <c r="C145" s="9"/>
       <c r="D145" s="8">
-        <v>46248.168571574075</v>
+        <v>46260.642762627314</v>
       </c>
       <c r="E145" s="9" t="s">
         <v>190</v>
@@ -10000,7 +10042,7 @@
       </c>
       <c r="C146" s="6"/>
       <c r="D146" s="5">
-        <v>46248.16857436343</v>
+        <v>46260.64276206019</v>
       </c>
       <c r="E146" s="6" t="s">
         <v>190</v>
@@ -10051,7 +10093,7 @@
       </c>
       <c r="C147" s="9"/>
       <c r="D147" s="8">
-        <v>46248.16857642361</v>
+        <v>46260.64276164352</v>
       </c>
       <c r="E147" s="9" t="s">
         <v>190</v>
@@ -10102,7 +10144,7 @@
       </c>
       <c r="C148" s="6"/>
       <c r="D148" s="5">
-        <v>46248.16856126157</v>
+        <v>46260.64276171297</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>190</v>

</xml_diff>